<commit_message>
Add high-paying SDE2 company lists
</commit_message>
<xml_diff>
--- a/companies.xlsx
+++ b/companies.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="companies" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'companies'!$A$1:$E$30</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,13 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -52,15 +61,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -132,6 +149,20 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompaniesTable" displayName="CompaniesTable" ref="A1:E30" headerRowCount="1">
+  <autoFilter ref="A1:E30"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="company"/>
+    <tableColumn id="2" name="career_url"/>
+    <tableColumn id="3" name="priority"/>
+    <tableColumn id="4" name="notes"/>
+    <tableColumn id="5" name="enabled"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -423,13 +454,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -461,106 +492,766 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/OpenAI</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Verified Ashby example; replace with your target company</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AI research/platform; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Cohere</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>LLM platform; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Perplexity</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AI search/retrieval; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Cursor</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AI coding/devtools; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>LangChain</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/LangChain</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Agent/RAG tooling; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Replit</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Replit</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>AI coding/platform; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>AI audio platform; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Runway</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Runway</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>GenAI media; verified Ashby</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/databricks</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Data/AI platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/stripe</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Backend/platform engineering; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Coinbase</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/coinbase</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Distributed systems/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Datadog</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/datadog</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Infra/observability/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/mongodb</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Database/search/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Elastic</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/elastic</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Search/retrieval/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/figma</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Collab/dev platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Roblox</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/roblox</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Large scale infra; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Affirm</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/affirm</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Backend/data/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Asana</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/asana</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Product/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Dropbox</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/dropbox</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Infra/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/instacart</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Backend/data; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/cloudflare</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Infra/distributed systems; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Okta</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/okta</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Identity/platform/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Twilio</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/twilio</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Comms platform/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Brex</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/brex</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Fintech/backend/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Rubrik</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/rubrik</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Cloud/data infra; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Samsara</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/samsara</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>IoT/platform/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/scaleai</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>AI data/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>https://boards.greenhouse.io/airbnb</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Large scale product/backend; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/reddit</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Verified Greenhouse example; replace with your target company</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Reddit</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/reddit</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Verified Greenhouse example; replace with your target company</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Databricks</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://boards.greenhouse.io/databricks</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Verified Greenhouse example; replace with your target company</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Search/feed/backend/platform; verified Greenhouse</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E30"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>